<commit_message>
fixe repetition encours 0
</commit_message>
<xml_diff>
--- a/PAMF_DIG F2 - monthly2026-07-15.xlsx
+++ b/PAMF_DIG F2 - monthly2026-07-15.xlsx
@@ -633,7 +633,7 @@
         <v>0.09</v>
       </c>
       <c r="N3" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -1363,7 +1363,7 @@
         <v>0.09</v>
       </c>
       <c r="N13" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -3626,7 +3626,7 @@
         <v>0.09</v>
       </c>
       <c r="N44" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -5305,7 +5305,7 @@
         <v>0.09</v>
       </c>
       <c r="N67" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -8152,7 +8152,7 @@
         <v>0.09</v>
       </c>
       <c r="N106" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>

</xml_diff>